<commit_message>
feat: implement association rule mining using Apriori algorithm and generate visualization assets
</commit_message>
<xml_diff>
--- a/hasil_barang_alfamaret.xlsx
+++ b/hasil_barang_alfamaret.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nama_barang" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="nama_barang" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -434,17 +422,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>struk_ke</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>tanggal_transaksi</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>nama_barang</t>
         </is>
@@ -452,46 +440,46 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NUVO WIPES</t>
+          <t>TROPICAL MYKPIL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SELECT BLT</t>
+          <t>ABC KCPMNS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NICE SOFT</t>
+          <t>you C APL</t>
         </is>
       </c>
     </row>
@@ -506,7 +494,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TROPICAL MYKPIL</t>
+          <t>YOU C LMN</t>
         </is>
       </c>
     </row>
@@ -521,352 +509,172 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ABC KCPMNS</t>
+          <t>TLR NG DC/PCS A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>you C APL</t>
+          <t>LEMNRL AIR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>YOU C LMN</t>
+          <t>SOSRO TWR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TLR NG DC/PCS A</t>
+          <t>SQ CSW</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LEMNRL AIR</t>
+          <t>SQ CHK ALMD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SOSRO TWR</t>
+          <t>CIMORY HZL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SOSRO TWR</t>
+          <t>CIMORY MTC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SQ CK CSW</t>
+          <t>FITMEUP PC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KNZLR SGL HT</t>
+          <t>AMUNIZER</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CIMORY NSM</t>
+          <t>ALFA ECOBGX</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SQ CSW</t>
+          <t>KNZLR SGL GJ</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SQ CHK ALMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>5</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CIMORY HZL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>CIMORY MTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>FITMEUP PC</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>AMUNIZER</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>ALFA ECOBGX</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>AQUVlVAAlR</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>FOREST GRP</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>7</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KNZLR SGL GJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>7</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
           <t>SQ BT ALMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>8</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>KNZLR SGL TYNG</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>8</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>KNZLR BKSGCJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>8</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>KNZLR SGL GJ</t>
         </is>
       </c>
     </row>

</xml_diff>